<commit_message>
ROI_Model: add bundled implementation scenario for Onboarding + Equipment
</commit_message>
<xml_diff>
--- a/data/Automation_Priority_Matrix.xlsx
+++ b/data/Automation_Priority_Matrix.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="225">
   <si>
     <t xml:space="preserve">Digital Workplace Automation Priority Model</t>
   </si>
@@ -597,6 +597,42 @@
   </si>
   <si>
     <t xml:space="preserve">Note: Onboarding and Equipment builds assume reuse of Micron's existing ServiceNow instance (per JD tool list), no separate licensing. Password Reset, Shift-Handoff, and Meeting Booking assume new dedicated tools with real published per-user/per-room pricing (see Assumptions tab). Shift-worker and room counts are synthetic subset estimates, flagged accordingly.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bundled Implementation Scenario (Onboarding + Equipment, same ServiceNow build)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Both builds are costed separately above ($30,000 each) as a conservative baseline. In practice, they share the same platform, admin team, and sprint (see Sprint_Backlog, Sprint 1), so combining them plausibly costs less than two independent builds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scenario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Onboarding One-Time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipment One-Time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Combined One-Time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3-Yr Combined Savings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Combined 3-Yr Net</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baseline (separate builds)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bundled (25% synergy discount, editable)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n/a (shared build)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25% is an editable planning assumption, not a sourced figure: it estimates shared discovery, ServiceNow admin setup, and testing effort. Adjust column D's formula input if your organization's actual shared-build savings differ.</t>
   </si>
   <si>
     <t xml:space="preserve">Sensitivity Analysis: How Fragile Is Each Ranking?</t>
@@ -858,7 +894,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -952,6 +988,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1260,11 +1300,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="95883391"/>
-        <c:axId val="69314740"/>
+        <c:axId val="2144573"/>
+        <c:axId val="20416525"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="95883391"/>
+        <c:axId val="2144573"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1330,7 +1370,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69314740"/>
+        <c:crossAx val="20416525"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1338,7 +1378,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="69314740"/>
+        <c:axId val="20416525"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1380,7 +1420,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95883391"/>
+        <c:crossAx val="2144573"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2761,7 +2801,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -3110,9 +3150,111 @@
       <c r="L13" s="20"/>
       <c r="M13" s="20"/>
     </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="20" t="s">
+        <v>192</v>
+      </c>
+      <c r="B16" s="20"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="20"/>
+      <c r="L16" s="20"/>
+      <c r="M16" s="20"/>
+    </row>
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B19" s="15" t="n">
+        <f aca="false">D5</f>
+        <v>30000</v>
+      </c>
+      <c r="C19" s="15" t="n">
+        <f aca="false">D7</f>
+        <v>30000</v>
+      </c>
+      <c r="D19" s="15" t="n">
+        <f aca="false">B19+C19</f>
+        <v>60000</v>
+      </c>
+      <c r="E19" s="15" t="n">
+        <f aca="false">(B5*3)+(B7*3)</f>
+        <v>349272</v>
+      </c>
+      <c r="F19" s="22" t="n">
+        <f aca="false">E19-D19</f>
+        <v>289272</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="D20" s="24" t="n">
+        <f aca="false">D19*(1-0.25)</f>
+        <v>45000</v>
+      </c>
+      <c r="E20" s="15" t="n">
+        <f aca="false">E19</f>
+        <v>349272</v>
+      </c>
+      <c r="F20" s="24" t="n">
+        <f aca="false">E20-D20</f>
+        <v>304272</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="20" t="s">
+        <v>202</v>
+      </c>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
+      <c r="F22" s="20"/>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
     <mergeCell ref="A13:M13"/>
+    <mergeCell ref="A16:M16"/>
+    <mergeCell ref="A22:F22"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3141,12 +3283,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3154,40 +3296,40 @@
         <v>41</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3235,7 +3377,7 @@
         <f aca="false">MAX(F5:K5)-MIN(F5:K5)</f>
         <v>13.3333333333333</v>
       </c>
-      <c r="M5" s="24" t="str">
+      <c r="M5" s="25" t="str">
         <f aca="false">IF(ABS(F5-G5)&gt;=ABS(H5-I5),IF(ABS(F5-G5)&gt;=ABS(J5-K5),"Feasibility","Risk"),IF(ABS(H5-I5)&gt;=ABS(J5-K5),"Impact","Risk"))</f>
         <v>Risk</v>
       </c>
@@ -3285,7 +3427,7 @@
         <f aca="false">MAX(F6:K6)-MIN(F6:K6)</f>
         <v>4.16666666666667</v>
       </c>
-      <c r="M6" s="24" t="str">
+      <c r="M6" s="25" t="str">
         <f aca="false">IF(ABS(F6-G6)&gt;=ABS(H6-I6),IF(ABS(F6-G6)&gt;=ABS(J6-K6),"Feasibility","Risk"),IF(ABS(H6-I6)&gt;=ABS(J6-K6),"Impact","Risk"))</f>
         <v>Risk</v>
       </c>
@@ -3335,7 +3477,7 @@
         <f aca="false">MAX(F7:K7)-MIN(F7:K7)</f>
         <v>12.5</v>
       </c>
-      <c r="M7" s="24" t="str">
+      <c r="M7" s="25" t="str">
         <f aca="false">IF(ABS(F7-G7)&gt;=ABS(H7-I7),IF(ABS(F7-G7)&gt;=ABS(J7-K7),"Feasibility","Risk"),IF(ABS(H7-I7)&gt;=ABS(J7-K7),"Impact","Risk"))</f>
         <v>Impact</v>
       </c>
@@ -3385,7 +3527,7 @@
         <f aca="false">MAX(F8:K8)-MIN(F8:K8)</f>
         <v>13.3333333333333</v>
       </c>
-      <c r="M8" s="24" t="str">
+      <c r="M8" s="25" t="str">
         <f aca="false">IF(ABS(F8-G8)&gt;=ABS(H8-I8),IF(ABS(F8-G8)&gt;=ABS(J8-K8),"Feasibility","Risk"),IF(ABS(H8-I8)&gt;=ABS(J8-K8),"Impact","Risk"))</f>
         <v>Risk</v>
       </c>
@@ -3435,14 +3577,14 @@
         <f aca="false">MAX(F9:K9)-MIN(F9:K9)</f>
         <v>10</v>
       </c>
-      <c r="M9" s="24" t="str">
+      <c r="M9" s="25" t="str">
         <f aca="false">IF(ABS(F9-G9)&gt;=ABS(H9-I9),IF(ABS(F9-G9)&gt;=ABS(J9-K9),"Feasibility","Risk"),IF(ABS(H9-I9)&gt;=ABS(J9-K9),"Impact","Risk"))</f>
         <v>Impact</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="20"/>
@@ -3459,23 +3601,23 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="B15" s="0" t="n">
         <f aca="false">F7</f>
@@ -3488,7 +3630,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="B16" s="0" t="n">
         <f aca="false">H7</f>
@@ -3501,7 +3643,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="B17" s="0" t="n">
         <f aca="false">J7</f>

</xml_diff>